<commit_message>
v13.35 — Recherche rapide d'un dossier sur le tableau de bord + page d'accueil en version mobile (menu burger, carrousels, barre d'action) + v13.33/v13.34
</commit_message>
<xml_diff>
--- a/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
+++ b/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
@@ -10,10 +10,10 @@
   <sheets>
     <sheet name="Paramètres" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Simulation commercial" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Rentabilité IDEAFORMA" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Rentabilité MY EASY AUTO" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Suivi prospects" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -110,7 +110,7 @@
     <t xml:space="preserve">Simulateur de commissions — apporteurs d'affaires My Easy Auto</t>
   </si>
   <si>
-    <t xml:space="preserve">Cellules JAUNES = à modifier. Tout le reste est calculé. Grille en vigueur au 1er septembre 2026 (IDEAFORMA).</t>
+    <t xml:space="preserve">Cellules JAUNES = à modifier. Tout le reste est calculé. Grille en vigueur au 1er septembre 2026 (MY EASY AUTO).</t>
   </si>
   <si>
     <t xml:space="preserve">Légende : jaune = hypothèse modifiable · bleu = valeur saisie · noir = formule</t>
@@ -122,19 +122,19 @@
     <t xml:space="preserve">Prix HT / mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Heures secrétariat</t>
+    <t xml:space="preserve">Heures Adhésion Service</t>
   </si>
   <si>
     <t xml:space="preserve">Prime de signature</t>
   </si>
   <si>
-    <t xml:space="preserve">Prime de fidélité (0 depuis la v1.2)</t>
+    <t xml:space="preserve">Prime de fidélité — supprimée (grille v1.2), laissée à 0</t>
   </si>
   <si>
     <t xml:space="preserve">Bonus engagement 12 mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Secrétaire / mois (heures × taux)</t>
+    <t xml:space="preserve">Chargé de mission / mois (heures × taux)</t>
   </si>
   <si>
     <t xml:space="preserve">Coût technique / mois</t>
@@ -143,13 +143,13 @@
     <t xml:space="preserve">ESSENTIEL</t>
   </si>
   <si>
-    <t xml:space="preserve">STARTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFORT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SÉRÉNITÉ</t>
+    <t xml:space="preserve">ADHÉSION SERVICE PLUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADHÉSION SERVICE PREMIUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADHÉSION SERVICE ULTIMATE</t>
   </si>
   <si>
     <t xml:space="preserve">Hypothèses générales</t>
@@ -158,7 +158,7 @@
     <t xml:space="preserve">Taux de conservation des garages à M6</t>
   </si>
   <si>
-    <t xml:space="preserve">Taux horaire versé à la secrétaire (€ HT / heure de forfait)</t>
+    <t xml:space="preserve">Taux horaire versé au chargé de mission (€ HT / heure de forfait)</t>
   </si>
   <si>
     <t xml:space="preserve">Coût technique par garage et par mois (hébergement, IA, emails)</t>
@@ -191,7 +191,7 @@
     <t xml:space="preserve">Palier 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Source des prix et du taux horaire : NOTE-STRATEGIE-TARIFAIRE et IDEAFORMA_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.3 du 27/08/2026 (une prime unique par garage ; versée dès la 1re mensualité si engagement 12 mois, à la 3e sinon ; reprise si arrêt avant 3 mensualités).</t>
+    <t xml:space="preserve">Source des prix et du taux horaire : NOTE-STRATEGIE-TARIFAIRE et MYEASYAUTO_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.3, en vigueur au 1er septembre 2026 (une prime unique par garage ; versée dès la 1re mensualité si engagement 12 mois, à la 3e sinon ; reprise si arrêt avant 3 mensualités).</t>
   </si>
   <si>
     <t xml:space="preserve">Ce que gagne le commercial selon son rythme</t>
@@ -224,7 +224,7 @@
     <t xml:space="preserve">Bonus engagement 12 mois (× part engagée)</t>
   </si>
   <si>
-    <t xml:space="preserve">Primes de fidélité (× taux de conservation)</t>
+    <t xml:space="preserve">Primes de fidélité — supprimées (grille v1.2), à 0</t>
   </si>
   <si>
     <t xml:space="preserve">Total généré par un mois de signatures</t>
@@ -245,7 +245,7 @@
     <t xml:space="preserve">Primes de signature + bonus engagement perçus</t>
   </si>
   <si>
-    <t xml:space="preserve">Primes de fidélité perçues</t>
+    <t xml:space="preserve">Primes de fidélité (supprimées, à 0)</t>
   </si>
   <si>
     <t xml:space="preserve">Bonus de volume</t>
@@ -266,7 +266,7 @@
     <t xml:space="preserve">Revenu mensuel moyen en croisière</t>
   </si>
   <si>
-    <t xml:space="preserve">Ce que rapporte un garage à IDEAFORMA, commissions comprises</t>
+    <t xml:space="preserve">Ce que rapporte un garage à MY EASY AUTO, commissions comprises</t>
   </si>
   <si>
     <t xml:space="preserve">Par formule, sur la première année (avec commission) puis en année 2 (sans commission). Toutes les hypothèses viennent de l'onglet Paramètres.</t>
@@ -278,7 +278,7 @@
     <t xml:space="preserve">Chiffre d'affaires HT (12 mois)</t>
   </si>
   <si>
-    <t xml:space="preserve">Secrétaire (heures × taux horaire)</t>
+    <t xml:space="preserve">Chargé de mission (heures × taux horaire)</t>
   </si>
   <si>
     <t xml:space="preserve">Coûts techniques</t>
@@ -287,7 +287,7 @@
     <t xml:space="preserve">Commission apporteur : signature + bonus engagement (× part engagée)</t>
   </si>
   <si>
-    <t xml:space="preserve">Commission apporteur : fidélité (× taux de conservation)</t>
+    <t xml:space="preserve">Commission apporteur : fidélité — supprimée, à 0</t>
   </si>
   <si>
     <t xml:space="preserve">Marge brute année 1 (avant coûts fixes et rémunération)</t>
@@ -302,7 +302,7 @@
     <t xml:space="preserve">Année 2 et suivantes — par garage</t>
   </si>
   <si>
-    <t xml:space="preserve">Secrétaire + coûts techniques</t>
+    <t xml:space="preserve">Chargé de mission + coûts techniques</t>
   </si>
   <si>
     <t xml:space="preserve">Marge brute année 2 (aucune commission)</t>
@@ -320,7 +320,7 @@
     <t xml:space="preserve">Marge brute récurrente en année 2 (× taux de conservation)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture : la commission représente environ un tiers de la marge brute de la première année sur les formules avec secrétariat, et rien ensuite. Les coûts fixes d'IDEAFORMA (~270 € / mois, cf. note stratégique) et la rémunération du dirigeant ne sont pas déduits ici.</t>
+    <t xml:space="preserve">Lecture : la commission représente environ 13 % de la marge brute de la première année sur les formules Adhésion Service, et rien ensuite. Les coûts fixes d'MY EASY AUTO (~270 € / mois, cf. note stratégique) et la rémunération du dirigeant ne sont pas déduits ici.</t>
   </si>
   <si>
     <t xml:space="preserve">Suivi des prospects — à envoyer chaque vendredi à contact@myeasyauto.fr</t>
@@ -419,7 +419,7 @@
     <t xml:space="preserve">Rappeler après la démo</t>
   </si>
   <si>
-    <t xml:space="preserve">Secrétaire partie en juin, 3 factures AXA &gt; 90 jours</t>
+    <t xml:space="preserve">Personne chargée de l'administratif partie en juin, 3 factures AXA &gt; 90 jours</t>
   </si>
   <si>
     <t xml:space="preserve">Garages contactés</t>
@@ -3881,7 +3881,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M200" type="list">
-      <formula1>"ESSENTIEL,STARTER,CONFORT,SÉRÉNITÉ"</formula1>
+      <formula1>"ESSENTIEL,ADHÉSION SERVICE PLUS,ADHÉSION SERVICE PREMIUM,ADHÉSION SERVICE ULTIMATE"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N5:N200" type="list">

</xml_diff>